<commit_message>
added skeleton of 2450 guidance
</commit_message>
<xml_diff>
--- a/docs/StructureDefinition-cibmtr-additional-peri-transplant-medication.xlsx
+++ b/docs/StructureDefinition-cibmtr-additional-peri-transplant-medication.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1749" uniqueCount="348">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1749" uniqueCount="347">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2022-09-08T13:29:45-05:00</t>
+    <t>2022-11-09T13:32:08-06:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -253,10 +253,6 @@
   </si>
   <si>
     <t>The US Core Medication Profile is based upon the core FHIR Medication Resource and created to meet the 2015 Edition Common Clinical Data Set 'Medications' requirements.</t>
-  </si>
-  <si>
-    <t>dom-2:If the resource is contained in another resource, it SHALL NOT contain nested Resources {contained.contained.empty()}
-dom-3:If the resource is contained in another resource, it SHALL be referred to from elsewhere in the resource or SHALL refer to the containing resource {contained.where((('#'+id in (%resource.descendants().reference | %resource.descendants().as(canonical) | %resource.descendants().as(uri) | %resource.descendants().as(url))) or descendants().where(reference = '#').exists() or descendants().where(as(canonical) = '#').exists() or descendants().where(as(canonical) = '#').exists()).not()).trace('unmatched', id).empty()}dom-4:If a resource is contained in another resource, it SHALL NOT have a meta.versionId or a meta.lastUpdated {contained.meta.versionId.empty() and contained.meta.lastUpdated.empty()}dom-5:If a resource is contained in another resource, it SHALL NOT have a security label {contained.meta.security.empty()}dom-6:A resource should have narrative for robust management {text.`div`.exists()}</t>
   </si>
   <si>
     <t>NewRx/MedicationPrescribed@@ -280,111 +276,111 @@
     <t>Y</t>
   </si>
   <si>
+    <t xml:space="preserve">id
+</t>
+  </si>
+  <si>
+    <t>Logical id of this artifact</t>
+  </si>
+  <si>
+    <t>The logical id of the resource, as used in the URL for the resource. Once assigned, this value never changes.</t>
+  </si>
+  <si>
+    <t>The only time that a resource does not have an id is when it is being submitted to the server using a create operation.</t>
+  </si>
+  <si>
+    <t>Resource.id</t>
+  </si>
+  <si>
+    <t>Medication.meta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meta
+</t>
+  </si>
+  <si>
+    <t>Metadata about the resource</t>
+  </si>
+  <si>
+    <t>The metadata about the resource. This is content that is maintained by the infrastructure. Changes to the content might not always be associated with version changes to the resource.</t>
+  </si>
+  <si>
+    <t>Resource.meta</t>
+  </si>
+  <si>
+    <t>Medication.meta.id</t>
+  </si>
+  <si>
     <t xml:space="preserve">string
 </t>
   </si>
   <si>
-    <t>Logical id of this artifact</t>
-  </si>
-  <si>
-    <t>The logical id of the resource, as used in the URL for the resource. Once assigned, this value never changes.</t>
-  </si>
-  <si>
-    <t>The only time that a resource does not have an id is when it is being submitted to the server using a create operation.</t>
-  </si>
-  <si>
-    <t>Resource.id</t>
-  </si>
-  <si>
-    <t>Medication.meta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Meta
+    <t>Unique id for inter-element referencing</t>
+  </si>
+  <si>
+    <t>Unique id for the element within a resource (for internal references). This may be any string value that does not contain spaces.</t>
+  </si>
+  <si>
+    <t>Element.id</t>
+  </si>
+  <si>
+    <t>n/a</t>
+  </si>
+  <si>
+    <t>Medication.meta.extension</t>
+  </si>
+  <si>
+    <t>extensions
+user content</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extension
 </t>
   </si>
   <si>
-    <t>Metadata about the resource</t>
-  </si>
-  <si>
-    <t>The metadata about the resource. This is content that is maintained by the infrastructure. Changes to the content might not always be associated with version changes to the resource.</t>
-  </si>
-  <si>
-    <t>Resource.meta</t>
+    <t>Additional content defined by implementations</t>
+  </si>
+  <si>
+    <t>May be used to represent additional information that is not part of the basic definition of the element. To make the use of extensions safe and manageable, there is a strict set of governance  applied to the definition and use of extensions. Though any implementer can define an extension, there is a set of requirements that SHALL be met as part of the definition of the extension.</t>
+  </si>
+  <si>
+    <t>There can be no stigma associated with the use of extensions by any application, project, or standard - regardless of the institution or jurisdiction that uses or defines the extensions.  The use of extensions is what allows the FHIR specification to retain a core level of simplicity for everyone.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">value:url}
+</t>
+  </si>
+  <si>
+    <t>Extensions are always sliced by (at least) url</t>
+  </si>
+  <si>
+    <t>open</t>
+  </si>
+  <si>
+    <t>Element.extension</t>
+  </si>
+  <si>
+    <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
+ext-1:Must have either extensions or value[x], not both {extension.exists() != value.exists()}</t>
+  </si>
+  <si>
+    <t>Medication.meta.versionId</t>
+  </si>
+  <si>
+    <t>Version specific identifier</t>
+  </si>
+  <si>
+    <t>The version specific identifier, as it appears in the version portion of the URL. This value changes when the resource is created, updated, or deleted.</t>
+  </si>
+  <si>
+    <t>The server assigns this value, and ignores what the client specifies, except in the case that the server is imposing version integrity on updates/deletes.</t>
+  </si>
+  <si>
+    <t>Meta.versionId</t>
   </si>
   <si>
     <t xml:space="preserve">ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
 </t>
-  </si>
-  <si>
-    <t>Medication.meta.id</t>
-  </si>
-  <si>
-    <t>Unique id for inter-element referencing</t>
-  </si>
-  <si>
-    <t>Unique id for the element within a resource (for internal references). This may be any string value that does not contain spaces.</t>
-  </si>
-  <si>
-    <t>Element.id</t>
-  </si>
-  <si>
-    <t>n/a</t>
-  </si>
-  <si>
-    <t>Medication.meta.extension</t>
-  </si>
-  <si>
-    <t>extensions
-user content</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extension
-</t>
-  </si>
-  <si>
-    <t>Additional content defined by implementations</t>
-  </si>
-  <si>
-    <t>May be used to represent additional information that is not part of the basic definition of the element. To make the use of extensions safe and manageable, there is a strict set of governance  applied to the definition and use of extensions. Though any implementer can define an extension, there is a set of requirements that SHALL be met as part of the definition of the extension.</t>
-  </si>
-  <si>
-    <t>There can be no stigma associated with the use of extensions by any application, project, or standard - regardless of the institution or jurisdiction that uses or defines the extensions.  The use of extensions is what allows the FHIR specification to retain a core level of simplicity for everyone.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">value:url}
-</t>
-  </si>
-  <si>
-    <t>Extensions are always sliced by (at least) url</t>
-  </si>
-  <si>
-    <t>open</t>
-  </si>
-  <si>
-    <t>Element.extension</t>
-  </si>
-  <si>
-    <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
-ext-1:Must have either extensions or value[x], not both {extension.exists() != value.exists()}</t>
-  </si>
-  <si>
-    <t>Medication.meta.versionId</t>
-  </si>
-  <si>
-    <t xml:space="preserve">id
-</t>
-  </si>
-  <si>
-    <t>Version specific identifier</t>
-  </si>
-  <si>
-    <t>The version specific identifier, as it appears in the version portion of the URL. This value changes when the resource is created, updated, or deleted.</t>
-  </si>
-  <si>
-    <t>The server assigns this value, and ignores what the client specifies, except in the case that the server is imposing version integrity on updates/deletes.</t>
-  </si>
-  <si>
-    <t>Meta.versionId</t>
   </si>
   <si>
     <t>Medication.meta.lastUpdated</t>
@@ -1677,13 +1673,13 @@
         <v>74</v>
       </c>
       <c r="AI2" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AJ2" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="AJ2" t="s" s="2">
+      <c r="AK2" t="s" s="2">
         <v>80</v>
-      </c>
-      <c r="AK2" t="s" s="2">
-        <v>81</v>
       </c>
       <c r="AL2" t="s" s="2">
         <v>74</v>
@@ -1694,7 +1690,7 @@
     </row>
     <row r="3" hidden="true">
       <c r="A3" t="s" s="2">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" t="s" s="2">
@@ -1705,28 +1701,28 @@
         <v>75</v>
       </c>
       <c r="F3" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="G3" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="H3" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="I3" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="G3" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="H3" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="I3" t="s" s="2">
+      <c r="J3" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="J3" t="s" s="2">
+      <c r="K3" t="s" s="2">
         <v>85</v>
       </c>
-      <c r="K3" t="s" s="2">
+      <c r="L3" t="s" s="2">
         <v>86</v>
       </c>
-      <c r="L3" t="s" s="2">
+      <c r="M3" t="s" s="2">
         <v>87</v>
-      </c>
-      <c r="M3" t="s" s="2">
-        <v>88</v>
       </c>
       <c r="N3" s="2"/>
       <c r="O3" t="s" s="2">
@@ -1776,13 +1772,13 @@
         <v>74</v>
       </c>
       <c r="AE3" t="s" s="2">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="AF3" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AG3" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AH3" t="s" s="2">
         <v>74</v>
@@ -1805,7 +1801,7 @@
     </row>
     <row r="4" hidden="true">
       <c r="A4" t="s" s="2">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" t="s" s="2">
@@ -1816,25 +1812,25 @@
         <v>75</v>
       </c>
       <c r="F4" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="G4" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="H4" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="I4" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="G4" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="H4" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="I4" t="s" s="2">
-        <v>84</v>
-      </c>
       <c r="J4" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="K4" t="s" s="2">
         <v>91</v>
       </c>
-      <c r="K4" t="s" s="2">
+      <c r="L4" t="s" s="2">
         <v>92</v>
-      </c>
-      <c r="L4" t="s" s="2">
-        <v>93</v>
       </c>
       <c r="M4" s="2"/>
       <c r="N4" s="2"/>
@@ -1885,19 +1881,19 @@
         <v>74</v>
       </c>
       <c r="AE4" t="s" s="2">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="AF4" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AG4" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AH4" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AI4" t="s" s="2">
-        <v>95</v>
+        <v>74</v>
       </c>
       <c r="AJ4" t="s" s="2">
         <v>74</v>
@@ -1914,7 +1910,7 @@
     </row>
     <row r="5" hidden="true">
       <c r="A5" t="s" s="2">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" t="s" s="2">
@@ -1925,7 +1921,7 @@
         <v>75</v>
       </c>
       <c r="F5" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G5" t="s" s="2">
         <v>74</v>
@@ -1937,13 +1933,13 @@
         <v>74</v>
       </c>
       <c r="J5" t="s" s="2">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="K5" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="L5" t="s" s="2">
         <v>97</v>
-      </c>
-      <c r="L5" t="s" s="2">
-        <v>98</v>
       </c>
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
@@ -1994,25 +1990,25 @@
         <v>74</v>
       </c>
       <c r="AE5" t="s" s="2">
+        <v>98</v>
+      </c>
+      <c r="AF5" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AG5" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AH5" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AI5" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AJ5" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AK5" t="s" s="2">
         <v>99</v>
-      </c>
-      <c r="AF5" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AG5" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH5" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AI5" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AJ5" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AK5" t="s" s="2">
-        <v>100</v>
       </c>
       <c r="AL5" t="s" s="2">
         <v>74</v>
@@ -2023,11 +2019,11 @@
     </row>
     <row r="6" hidden="true">
       <c r="A6" t="s" s="2">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" t="s" s="2">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" t="s" s="2">
@@ -2046,16 +2042,16 @@
         <v>74</v>
       </c>
       <c r="J6" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="K6" t="s" s="2">
         <v>103</v>
       </c>
-      <c r="K6" t="s" s="2">
+      <c r="L6" t="s" s="2">
         <v>104</v>
       </c>
-      <c r="L6" t="s" s="2">
+      <c r="M6" t="s" s="2">
         <v>105</v>
-      </c>
-      <c r="M6" t="s" s="2">
-        <v>106</v>
       </c>
       <c r="N6" s="2"/>
       <c r="O6" t="s" s="2">
@@ -2093,19 +2089,19 @@
         <v>74</v>
       </c>
       <c r="AA6" t="s" s="2">
+        <v>106</v>
+      </c>
+      <c r="AB6" t="s" s="2">
         <v>107</v>
       </c>
-      <c r="AB6" t="s" s="2">
+      <c r="AC6" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AD6" t="s" s="2">
         <v>108</v>
       </c>
-      <c r="AC6" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AD6" t="s" s="2">
+      <c r="AE6" t="s" s="2">
         <v>109</v>
-      </c>
-      <c r="AE6" t="s" s="2">
-        <v>110</v>
       </c>
       <c r="AF6" t="s" s="2">
         <v>75</v>
@@ -2117,13 +2113,13 @@
         <v>74</v>
       </c>
       <c r="AI6" t="s" s="2">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AJ6" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AK6" t="s" s="2">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="AL6" t="s" s="2">
         <v>74</v>
@@ -2134,7 +2130,7 @@
     </row>
     <row r="7" hidden="true">
       <c r="A7" t="s" s="2">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" t="s" s="2">
@@ -2145,28 +2141,28 @@
         <v>75</v>
       </c>
       <c r="F7" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="G7" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="H7" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="I7" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="G7" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="H7" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="I7" t="s" s="2">
+      <c r="J7" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="J7" t="s" s="2">
+      <c r="K7" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="L7" t="s" s="2">
         <v>113</v>
       </c>
-      <c r="K7" t="s" s="2">
+      <c r="M7" t="s" s="2">
         <v>114</v>
-      </c>
-      <c r="L7" t="s" s="2">
-        <v>115</v>
-      </c>
-      <c r="M7" t="s" s="2">
-        <v>116</v>
       </c>
       <c r="N7" s="2"/>
       <c r="O7" t="s" s="2">
@@ -2216,19 +2212,19 @@
         <v>74</v>
       </c>
       <c r="AE7" t="s" s="2">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="AF7" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AG7" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AH7" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AI7" t="s" s="2">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="AJ7" t="s" s="2">
         <v>74</v>
@@ -2245,7 +2241,7 @@
     </row>
     <row r="8" hidden="true">
       <c r="A8" t="s" s="2">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" t="s" s="2">
@@ -2256,28 +2252,28 @@
         <v>75</v>
       </c>
       <c r="F8" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="G8" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="H8" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="I8" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="G8" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="H8" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="I8" t="s" s="2">
-        <v>84</v>
-      </c>
       <c r="J8" t="s" s="2">
+        <v>118</v>
+      </c>
+      <c r="K8" t="s" s="2">
         <v>119</v>
       </c>
-      <c r="K8" t="s" s="2">
+      <c r="L8" t="s" s="2">
         <v>120</v>
       </c>
-      <c r="L8" t="s" s="2">
+      <c r="M8" t="s" s="2">
         <v>121</v>
-      </c>
-      <c r="M8" t="s" s="2">
-        <v>122</v>
       </c>
       <c r="N8" s="2"/>
       <c r="O8" t="s" s="2">
@@ -2327,19 +2323,19 @@
         <v>74</v>
       </c>
       <c r="AE8" t="s" s="2">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="AF8" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AG8" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AH8" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AI8" t="s" s="2">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="AJ8" t="s" s="2">
         <v>74</v>
@@ -2356,7 +2352,7 @@
     </row>
     <row r="9" hidden="true">
       <c r="A9" t="s" s="2">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" t="s" s="2">
@@ -2367,28 +2363,28 @@
         <v>75</v>
       </c>
       <c r="F9" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="G9" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="H9" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="I9" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="G9" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="H9" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="I9" t="s" s="2">
-        <v>84</v>
-      </c>
       <c r="J9" t="s" s="2">
+        <v>124</v>
+      </c>
+      <c r="K9" t="s" s="2">
         <v>125</v>
       </c>
-      <c r="K9" t="s" s="2">
+      <c r="L9" t="s" s="2">
         <v>126</v>
       </c>
-      <c r="L9" t="s" s="2">
+      <c r="M9" t="s" s="2">
         <v>127</v>
-      </c>
-      <c r="M9" t="s" s="2">
-        <v>128</v>
       </c>
       <c r="N9" s="2"/>
       <c r="O9" t="s" s="2">
@@ -2438,19 +2434,19 @@
         <v>74</v>
       </c>
       <c r="AE9" t="s" s="2">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="AF9" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AG9" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AH9" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AI9" t="s" s="2">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="AJ9" t="s" s="2">
         <v>74</v>
@@ -2467,7 +2463,7 @@
     </row>
     <row r="10" hidden="true">
       <c r="A10" t="s" s="2">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" t="s" s="2">
@@ -2487,19 +2483,19 @@
         <v>74</v>
       </c>
       <c r="I10" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J10" t="s" s="2">
+        <v>130</v>
+      </c>
+      <c r="K10" t="s" s="2">
         <v>131</v>
       </c>
-      <c r="K10" t="s" s="2">
+      <c r="L10" t="s" s="2">
         <v>132</v>
       </c>
-      <c r="L10" t="s" s="2">
+      <c r="M10" t="s" s="2">
         <v>133</v>
-      </c>
-      <c r="M10" t="s" s="2">
-        <v>134</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" t="s" s="2">
@@ -2549,7 +2545,7 @@
         <v>74</v>
       </c>
       <c r="AE10" t="s" s="2">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="AF10" t="s" s="2">
         <v>75</v>
@@ -2561,7 +2557,7 @@
         <v>74</v>
       </c>
       <c r="AI10" t="s" s="2">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="AJ10" t="s" s="2">
         <v>74</v>
@@ -2578,7 +2574,7 @@
     </row>
     <row r="11" hidden="true">
       <c r="A11" t="s" s="2">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" t="s" s="2">
@@ -2586,7 +2582,7 @@
       </c>
       <c r="D11" s="2"/>
       <c r="E11" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F11" t="s" s="2">
         <v>76</v>
@@ -2598,19 +2594,19 @@
         <v>74</v>
       </c>
       <c r="I11" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J11" t="s" s="2">
+        <v>136</v>
+      </c>
+      <c r="K11" t="s" s="2">
         <v>137</v>
       </c>
-      <c r="K11" t="s" s="2">
+      <c r="L11" t="s" s="2">
         <v>138</v>
       </c>
-      <c r="L11" t="s" s="2">
+      <c r="M11" t="s" s="2">
         <v>139</v>
-      </c>
-      <c r="M11" t="s" s="2">
-        <v>140</v>
       </c>
       <c r="N11" s="2"/>
       <c r="O11" t="s" s="2">
@@ -2636,31 +2632,31 @@
         <v>74</v>
       </c>
       <c r="W11" t="s" s="2">
+        <v>140</v>
+      </c>
+      <c r="X11" t="s" s="2">
         <v>141</v>
       </c>
-      <c r="X11" t="s" s="2">
+      <c r="Y11" t="s" s="2">
         <v>142</v>
       </c>
-      <c r="Y11" t="s" s="2">
+      <c r="Z11" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AA11" t="s" s="2">
         <v>143</v>
       </c>
-      <c r="Z11" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AA11" t="s" s="2">
+      <c r="AB11" t="s" s="2">
         <v>144</v>
       </c>
-      <c r="AB11" t="s" s="2">
+      <c r="AC11" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AD11" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="AE11" t="s" s="2">
         <v>145</v>
-      </c>
-      <c r="AC11" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AD11" t="s" s="2">
-        <v>109</v>
-      </c>
-      <c r="AE11" t="s" s="2">
-        <v>146</v>
       </c>
       <c r="AF11" t="s" s="2">
         <v>75</v>
@@ -2672,7 +2668,7 @@
         <v>74</v>
       </c>
       <c r="AI11" t="s" s="2">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="AJ11" t="s" s="2">
         <v>74</v>
@@ -2689,41 +2685,41 @@
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C12" t="s" s="2">
         <v>74</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="F12" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="G12" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="F12" t="s" s="2">
+      <c r="H12" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="I12" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="G12" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="H12" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="I12" t="s" s="2">
-        <v>84</v>
-      </c>
       <c r="J12" t="s" s="2">
+        <v>136</v>
+      </c>
+      <c r="K12" t="s" s="2">
         <v>137</v>
       </c>
-      <c r="K12" t="s" s="2">
+      <c r="L12" t="s" s="2">
         <v>138</v>
       </c>
-      <c r="L12" t="s" s="2">
+      <c r="M12" t="s" s="2">
         <v>139</v>
-      </c>
-      <c r="M12" t="s" s="2">
-        <v>140</v>
       </c>
       <c r="N12" s="2"/>
       <c r="O12" t="s" s="2">
@@ -2749,14 +2745,14 @@
         <v>74</v>
       </c>
       <c r="W12" t="s" s="2">
+        <v>140</v>
+      </c>
+      <c r="X12" t="s" s="2">
         <v>141</v>
       </c>
-      <c r="X12" t="s" s="2">
+      <c r="Y12" t="s" s="2">
         <v>142</v>
       </c>
-      <c r="Y12" t="s" s="2">
-        <v>143</v>
-      </c>
       <c r="Z12" t="s" s="2">
         <v>74</v>
       </c>
@@ -2773,7 +2769,7 @@
         <v>74</v>
       </c>
       <c r="AE12" t="s" s="2">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="AF12" t="s" s="2">
         <v>75</v>
@@ -2785,7 +2781,7 @@
         <v>74</v>
       </c>
       <c r="AI12" t="s" s="2">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="AJ12" t="s" s="2">
         <v>74</v>
@@ -2802,7 +2798,7 @@
     </row>
     <row r="13" hidden="true">
       <c r="A13" t="s" s="2">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" t="s" s="2">
@@ -2813,7 +2809,7 @@
         <v>75</v>
       </c>
       <c r="F13" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G13" t="s" s="2">
         <v>74</v>
@@ -2825,13 +2821,13 @@
         <v>74</v>
       </c>
       <c r="J13" t="s" s="2">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="K13" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="L13" t="s" s="2">
         <v>97</v>
-      </c>
-      <c r="L13" t="s" s="2">
-        <v>98</v>
       </c>
       <c r="M13" s="2"/>
       <c r="N13" s="2"/>
@@ -2882,25 +2878,25 @@
         <v>74</v>
       </c>
       <c r="AE13" t="s" s="2">
+        <v>98</v>
+      </c>
+      <c r="AF13" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AG13" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AH13" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AI13" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AJ13" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AK13" t="s" s="2">
         <v>99</v>
-      </c>
-      <c r="AF13" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AG13" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH13" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AI13" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AJ13" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AK13" t="s" s="2">
-        <v>100</v>
       </c>
       <c r="AL13" t="s" s="2">
         <v>74</v>
@@ -2911,11 +2907,11 @@
     </row>
     <row r="14" hidden="true">
       <c r="A14" t="s" s="2">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" t="s" s="2">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" t="s" s="2">
@@ -2934,16 +2930,16 @@
         <v>74</v>
       </c>
       <c r="J14" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="K14" t="s" s="2">
         <v>103</v>
       </c>
-      <c r="K14" t="s" s="2">
+      <c r="L14" t="s" s="2">
         <v>104</v>
       </c>
-      <c r="L14" t="s" s="2">
+      <c r="M14" t="s" s="2">
         <v>105</v>
-      </c>
-      <c r="M14" t="s" s="2">
-        <v>106</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" t="s" s="2">
@@ -2981,19 +2977,19 @@
         <v>74</v>
       </c>
       <c r="AA14" t="s" s="2">
+        <v>106</v>
+      </c>
+      <c r="AB14" t="s" s="2">
         <v>107</v>
       </c>
-      <c r="AB14" t="s" s="2">
+      <c r="AC14" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AD14" t="s" s="2">
         <v>108</v>
       </c>
-      <c r="AC14" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AD14" t="s" s="2">
+      <c r="AE14" t="s" s="2">
         <v>109</v>
-      </c>
-      <c r="AE14" t="s" s="2">
-        <v>110</v>
       </c>
       <c r="AF14" t="s" s="2">
         <v>75</v>
@@ -3005,13 +3001,13 @@
         <v>74</v>
       </c>
       <c r="AI14" t="s" s="2">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AJ14" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AK14" t="s" s="2">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="AL14" t="s" s="2">
         <v>74</v>
@@ -3022,7 +3018,7 @@
     </row>
     <row r="15" hidden="true">
       <c r="A15" t="s" s="2">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" t="s" s="2">
@@ -3030,34 +3026,34 @@
       </c>
       <c r="D15" s="2"/>
       <c r="E15" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="F15" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="G15" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="H15" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="I15" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="F15" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="G15" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="H15" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="I15" t="s" s="2">
-        <v>84</v>
-      </c>
       <c r="J15" t="s" s="2">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="K15" t="s" s="2">
+        <v>150</v>
+      </c>
+      <c r="L15" t="s" s="2">
         <v>151</v>
       </c>
-      <c r="L15" t="s" s="2">
+      <c r="M15" t="s" s="2">
         <v>152</v>
       </c>
-      <c r="M15" t="s" s="2">
+      <c r="N15" t="s" s="2">
         <v>153</v>
-      </c>
-      <c r="N15" t="s" s="2">
-        <v>154</v>
       </c>
       <c r="O15" t="s" s="2">
         <v>74</v>
@@ -3067,75 +3063,75 @@
         <v>74</v>
       </c>
       <c r="R15" t="s" s="2">
+        <v>154</v>
+      </c>
+      <c r="S15" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="T15" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="U15" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="V15" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="W15" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="X15" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="Y15" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="Z15" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AA15" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AB15" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AC15" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AD15" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AE15" t="s" s="2">
         <v>155</v>
       </c>
-      <c r="S15" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="T15" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="U15" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="V15" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="W15" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="X15" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Y15" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Z15" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AA15" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AB15" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AC15" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AD15" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AE15" t="s" s="2">
+      <c r="AF15" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AG15" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AH15" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AI15" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="AJ15" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AK15" t="s" s="2">
         <v>156</v>
       </c>
-      <c r="AF15" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AG15" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH15" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AI15" t="s" s="2">
-        <v>95</v>
-      </c>
-      <c r="AJ15" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AK15" t="s" s="2">
+      <c r="AL15" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AM15" t="s" s="2">
         <v>157</v>
-      </c>
-      <c r="AL15" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AM15" t="s" s="2">
-        <v>158</v>
       </c>
     </row>
     <row r="16" hidden="true">
       <c r="A16" t="s" s="2">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" t="s" s="2">
@@ -3146,28 +3142,28 @@
         <v>75</v>
       </c>
       <c r="F16" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="G16" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="H16" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="I16" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="G16" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="H16" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="I16" t="s" s="2">
-        <v>84</v>
-      </c>
       <c r="J16" t="s" s="2">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="K16" t="s" s="2">
+        <v>159</v>
+      </c>
+      <c r="L16" t="s" s="2">
         <v>160</v>
       </c>
-      <c r="L16" t="s" s="2">
+      <c r="M16" t="s" s="2">
         <v>161</v>
-      </c>
-      <c r="M16" t="s" s="2">
-        <v>162</v>
       </c>
       <c r="N16" s="2"/>
       <c r="O16" t="s" s="2">
@@ -3217,36 +3213,36 @@
         <v>74</v>
       </c>
       <c r="AE16" t="s" s="2">
+        <v>162</v>
+      </c>
+      <c r="AF16" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AG16" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AH16" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AI16" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="AJ16" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AK16" t="s" s="2">
         <v>163</v>
       </c>
-      <c r="AF16" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AG16" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH16" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AI16" t="s" s="2">
-        <v>95</v>
-      </c>
-      <c r="AJ16" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AK16" t="s" s="2">
+      <c r="AL16" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AM16" t="s" s="2">
         <v>164</v>
-      </c>
-      <c r="AL16" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AM16" t="s" s="2">
-        <v>165</v>
       </c>
     </row>
     <row r="17" hidden="true">
       <c r="A17" t="s" s="2">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" t="s" s="2">
@@ -3254,32 +3250,32 @@
       </c>
       <c r="D17" s="2"/>
       <c r="E17" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="F17" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="G17" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="H17" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="I17" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="F17" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="G17" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="H17" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="I17" t="s" s="2">
-        <v>84</v>
-      </c>
       <c r="J17" t="s" s="2">
+        <v>166</v>
+      </c>
+      <c r="K17" t="s" s="2">
         <v>167</v>
       </c>
-      <c r="K17" t="s" s="2">
+      <c r="L17" t="s" s="2">
         <v>168</v>
-      </c>
-      <c r="L17" t="s" s="2">
-        <v>169</v>
       </c>
       <c r="M17" s="2"/>
       <c r="N17" t="s" s="2">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="O17" t="s" s="2">
         <v>74</v>
@@ -3328,36 +3324,36 @@
         <v>74</v>
       </c>
       <c r="AE17" t="s" s="2">
+        <v>170</v>
+      </c>
+      <c r="AF17" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AG17" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AH17" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AI17" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="AJ17" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AK17" t="s" s="2">
         <v>171</v>
       </c>
-      <c r="AF17" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AG17" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH17" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AI17" t="s" s="2">
-        <v>95</v>
-      </c>
-      <c r="AJ17" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AK17" t="s" s="2">
+      <c r="AL17" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AM17" t="s" s="2">
         <v>172</v>
-      </c>
-      <c r="AL17" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AM17" t="s" s="2">
-        <v>173</v>
       </c>
     </row>
     <row r="18" hidden="true">
       <c r="A18" t="s" s="2">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" t="s" s="2">
@@ -3368,29 +3364,29 @@
         <v>75</v>
       </c>
       <c r="F18" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="G18" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="H18" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="I18" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="G18" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="H18" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="I18" t="s" s="2">
-        <v>84</v>
-      </c>
       <c r="J18" t="s" s="2">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="K18" t="s" s="2">
+        <v>174</v>
+      </c>
+      <c r="L18" t="s" s="2">
         <v>175</v>
-      </c>
-      <c r="L18" t="s" s="2">
-        <v>176</v>
       </c>
       <c r="M18" s="2"/>
       <c r="N18" t="s" s="2">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="O18" t="s" s="2">
         <v>74</v>
@@ -3439,36 +3435,36 @@
         <v>74</v>
       </c>
       <c r="AE18" t="s" s="2">
+        <v>177</v>
+      </c>
+      <c r="AF18" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AG18" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AH18" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AI18" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="AJ18" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AK18" t="s" s="2">
         <v>178</v>
       </c>
-      <c r="AF18" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AG18" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH18" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AI18" t="s" s="2">
-        <v>95</v>
-      </c>
-      <c r="AJ18" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AK18" t="s" s="2">
+      <c r="AL18" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AM18" t="s" s="2">
         <v>179</v>
-      </c>
-      <c r="AL18" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AM18" t="s" s="2">
-        <v>180</v>
       </c>
     </row>
     <row r="19" hidden="true">
       <c r="A19" t="s" s="2">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" t="s" s="2">
@@ -3479,31 +3475,31 @@
         <v>75</v>
       </c>
       <c r="F19" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="G19" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="H19" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="I19" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="G19" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="H19" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="I19" t="s" s="2">
-        <v>84</v>
-      </c>
       <c r="J19" t="s" s="2">
+        <v>181</v>
+      </c>
+      <c r="K19" t="s" s="2">
         <v>182</v>
       </c>
-      <c r="K19" t="s" s="2">
+      <c r="L19" t="s" s="2">
         <v>183</v>
       </c>
-      <c r="L19" t="s" s="2">
+      <c r="M19" t="s" s="2">
         <v>184</v>
       </c>
-      <c r="M19" t="s" s="2">
+      <c r="N19" t="s" s="2">
         <v>185</v>
-      </c>
-      <c r="N19" t="s" s="2">
-        <v>186</v>
       </c>
       <c r="O19" t="s" s="2">
         <v>74</v>
@@ -3552,36 +3548,36 @@
         <v>74</v>
       </c>
       <c r="AE19" t="s" s="2">
+        <v>186</v>
+      </c>
+      <c r="AF19" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AG19" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AH19" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AI19" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="AJ19" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AK19" t="s" s="2">
         <v>187</v>
       </c>
-      <c r="AF19" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AG19" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH19" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AI19" t="s" s="2">
-        <v>95</v>
-      </c>
-      <c r="AJ19" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AK19" t="s" s="2">
+      <c r="AL19" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AM19" t="s" s="2">
         <v>188</v>
-      </c>
-      <c r="AL19" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AM19" t="s" s="2">
-        <v>189</v>
       </c>
     </row>
     <row r="20" hidden="true">
       <c r="A20" t="s" s="2">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" t="s" s="2">
@@ -3601,19 +3597,19 @@
         <v>74</v>
       </c>
       <c r="I20" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J20" t="s" s="2">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="K20" t="s" s="2">
+        <v>190</v>
+      </c>
+      <c r="L20" t="s" s="2">
         <v>191</v>
       </c>
-      <c r="L20" t="s" s="2">
+      <c r="M20" t="s" s="2">
         <v>192</v>
-      </c>
-      <c r="M20" t="s" s="2">
-        <v>193</v>
       </c>
       <c r="N20" s="2"/>
       <c r="O20" t="s" s="2">
@@ -3639,31 +3635,31 @@
         <v>74</v>
       </c>
       <c r="W20" t="s" s="2">
+        <v>193</v>
+      </c>
+      <c r="X20" t="s" s="2">
         <v>194</v>
       </c>
-      <c r="X20" t="s" s="2">
+      <c r="Y20" t="s" s="2">
         <v>195</v>
       </c>
-      <c r="Y20" t="s" s="2">
+      <c r="Z20" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AA20" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AB20" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AC20" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AD20" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AE20" t="s" s="2">
         <v>196</v>
-      </c>
-      <c r="Z20" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AA20" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AB20" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AC20" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AD20" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AE20" t="s" s="2">
-        <v>197</v>
       </c>
       <c r="AF20" t="s" s="2">
         <v>75</v>
@@ -3675,7 +3671,7 @@
         <v>74</v>
       </c>
       <c r="AI20" t="s" s="2">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="AJ20" t="s" s="2">
         <v>74</v>
@@ -3692,7 +3688,7 @@
     </row>
     <row r="21" hidden="true">
       <c r="A21" t="s" s="2">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" t="s" s="2">
@@ -3703,28 +3699,28 @@
         <v>75</v>
       </c>
       <c r="F21" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="G21" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="H21" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="G21" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="H21" t="s" s="2">
-        <v>84</v>
-      </c>
       <c r="I21" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J21" t="s" s="2">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="K21" t="s" s="2">
+        <v>198</v>
+      </c>
+      <c r="L21" t="s" s="2">
         <v>199</v>
       </c>
-      <c r="L21" t="s" s="2">
+      <c r="M21" t="s" s="2">
         <v>200</v>
-      </c>
-      <c r="M21" t="s" s="2">
-        <v>201</v>
       </c>
       <c r="N21" s="2"/>
       <c r="O21" t="s" s="2">
@@ -3774,19 +3770,19 @@
         <v>74</v>
       </c>
       <c r="AE21" t="s" s="2">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AF21" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AG21" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AH21" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AI21" t="s" s="2">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="AJ21" t="s" s="2">
         <v>74</v>
@@ -3803,7 +3799,7 @@
     </row>
     <row r="22" hidden="true">
       <c r="A22" t="s" s="2">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" t="s" s="2">
@@ -3814,7 +3810,7 @@
         <v>75</v>
       </c>
       <c r="F22" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G22" t="s" s="2">
         <v>74</v>
@@ -3826,16 +3822,16 @@
         <v>74</v>
       </c>
       <c r="J22" t="s" s="2">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K22" t="s" s="2">
+        <v>203</v>
+      </c>
+      <c r="L22" t="s" s="2">
         <v>204</v>
       </c>
-      <c r="L22" t="s" s="2">
+      <c r="M22" t="s" s="2">
         <v>205</v>
-      </c>
-      <c r="M22" t="s" s="2">
-        <v>206</v>
       </c>
       <c r="N22" s="2"/>
       <c r="O22" t="s" s="2">
@@ -3861,43 +3857,43 @@
         <v>74</v>
       </c>
       <c r="W22" t="s" s="2">
+        <v>206</v>
+      </c>
+      <c r="X22" t="s" s="2">
         <v>207</v>
       </c>
-      <c r="X22" t="s" s="2">
+      <c r="Y22" t="s" s="2">
         <v>208</v>
       </c>
-      <c r="Y22" t="s" s="2">
+      <c r="Z22" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AA22" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AB22" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AC22" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AD22" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AE22" t="s" s="2">
         <v>209</v>
       </c>
-      <c r="Z22" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AA22" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AB22" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AC22" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AD22" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AE22" t="s" s="2">
-        <v>210</v>
-      </c>
       <c r="AF22" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AG22" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AH22" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AI22" t="s" s="2">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="AJ22" t="s" s="2">
         <v>74</v>
@@ -3914,18 +3910,18 @@
     </row>
     <row r="23" hidden="true">
       <c r="A23" t="s" s="2">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B23" s="2"/>
       <c r="C23" t="s" s="2">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D23" s="2"/>
       <c r="E23" t="s" s="2">
         <v>75</v>
       </c>
       <c r="F23" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G23" t="s" s="2">
         <v>74</v>
@@ -3937,16 +3933,16 @@
         <v>74</v>
       </c>
       <c r="J23" t="s" s="2">
+        <v>212</v>
+      </c>
+      <c r="K23" t="s" s="2">
         <v>213</v>
       </c>
-      <c r="K23" t="s" s="2">
+      <c r="L23" t="s" s="2">
         <v>214</v>
       </c>
-      <c r="L23" t="s" s="2">
+      <c r="M23" t="s" s="2">
         <v>215</v>
-      </c>
-      <c r="M23" t="s" s="2">
-        <v>216</v>
       </c>
       <c r="N23" s="2"/>
       <c r="O23" t="s" s="2">
@@ -3996,25 +3992,25 @@
         <v>74</v>
       </c>
       <c r="AE23" t="s" s="2">
+        <v>216</v>
+      </c>
+      <c r="AF23" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AG23" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AH23" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AI23" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="AJ23" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AK23" t="s" s="2">
         <v>217</v>
-      </c>
-      <c r="AF23" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AG23" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH23" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AI23" t="s" s="2">
-        <v>95</v>
-      </c>
-      <c r="AJ23" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AK23" t="s" s="2">
-        <v>218</v>
       </c>
       <c r="AL23" t="s" s="2">
         <v>74</v>
@@ -4025,11 +4021,11 @@
     </row>
     <row r="24" hidden="true">
       <c r="A24" t="s" s="2">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" t="s" s="2">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D24" s="2"/>
       <c r="E24" t="s" s="2">
@@ -4048,16 +4044,16 @@
         <v>74</v>
       </c>
       <c r="J24" t="s" s="2">
+        <v>220</v>
+      </c>
+      <c r="K24" t="s" s="2">
         <v>221</v>
       </c>
-      <c r="K24" t="s" s="2">
+      <c r="L24" t="s" s="2">
         <v>222</v>
       </c>
-      <c r="L24" t="s" s="2">
+      <c r="M24" t="s" s="2">
         <v>223</v>
-      </c>
-      <c r="M24" t="s" s="2">
-        <v>224</v>
       </c>
       <c r="N24" s="2"/>
       <c r="O24" t="s" s="2">
@@ -4107,7 +4103,7 @@
         <v>74</v>
       </c>
       <c r="AE24" t="s" s="2">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="AF24" t="s" s="2">
         <v>75</v>
@@ -4125,7 +4121,7 @@
         <v>74</v>
       </c>
       <c r="AK24" t="s" s="2">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="AL24" t="s" s="2">
         <v>74</v>
@@ -4136,11 +4132,11 @@
     </row>
     <row r="25" hidden="true">
       <c r="A25" t="s" s="2">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B25" s="2"/>
       <c r="C25" t="s" s="2">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D25" s="2"/>
       <c r="E25" t="s" s="2">
@@ -4159,16 +4155,16 @@
         <v>74</v>
       </c>
       <c r="J25" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="K25" t="s" s="2">
         <v>103</v>
       </c>
-      <c r="K25" t="s" s="2">
-        <v>104</v>
-      </c>
       <c r="L25" t="s" s="2">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="N25" s="2"/>
       <c r="O25" t="s" s="2">
@@ -4218,7 +4214,7 @@
         <v>74</v>
       </c>
       <c r="AE25" t="s" s="2">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="AF25" t="s" s="2">
         <v>75</v>
@@ -4230,13 +4226,13 @@
         <v>74</v>
       </c>
       <c r="AI25" t="s" s="2">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AJ25" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AK25" t="s" s="2">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="AL25" t="s" s="2">
         <v>74</v>
@@ -4247,11 +4243,11 @@
     </row>
     <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B26" s="2"/>
       <c r="C26" t="s" s="2">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D26" s="2"/>
       <c r="E26" t="s" s="2">
@@ -4264,25 +4260,25 @@
         <v>74</v>
       </c>
       <c r="H26" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I26" t="s" s="2">
         <v>74</v>
       </c>
       <c r="J26" t="s" s="2">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="K26" t="s" s="2">
+        <v>230</v>
+      </c>
+      <c r="L26" t="s" s="2">
         <v>231</v>
       </c>
-      <c r="L26" t="s" s="2">
+      <c r="M26" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="N26" t="s" s="2">
         <v>232</v>
-      </c>
-      <c r="M26" t="s" s="2">
-        <v>106</v>
-      </c>
-      <c r="N26" t="s" s="2">
-        <v>233</v>
       </c>
       <c r="O26" t="s" s="2">
         <v>74</v>
@@ -4331,7 +4327,7 @@
         <v>74</v>
       </c>
       <c r="AE26" t="s" s="2">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="AF26" t="s" s="2">
         <v>75</v>
@@ -4343,13 +4339,13 @@
         <v>74</v>
       </c>
       <c r="AI26" t="s" s="2">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AJ26" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AK26" t="s" s="2">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="AL26" t="s" s="2">
         <v>74</v>
@@ -4360,7 +4356,7 @@
     </row>
     <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" t="s" s="2">
@@ -4380,19 +4376,19 @@
         <v>74</v>
       </c>
       <c r="I27" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J27" t="s" s="2">
+        <v>235</v>
+      </c>
+      <c r="K27" t="s" s="2">
         <v>236</v>
       </c>
-      <c r="K27" t="s" s="2">
+      <c r="L27" t="s" s="2">
         <v>237</v>
       </c>
-      <c r="L27" t="s" s="2">
+      <c r="M27" t="s" s="2">
         <v>238</v>
-      </c>
-      <c r="M27" t="s" s="2">
-        <v>239</v>
       </c>
       <c r="N27" s="2"/>
       <c r="O27" t="s" s="2">
@@ -4442,7 +4438,7 @@
         <v>74</v>
       </c>
       <c r="AE27" t="s" s="2">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="AF27" t="s" s="2">
         <v>75</v>
@@ -4454,16 +4450,16 @@
         <v>74</v>
       </c>
       <c r="AI27" t="s" s="2">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="AJ27" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AK27" t="s" s="2">
+        <v>239</v>
+      </c>
+      <c r="AL27" t="s" s="2">
         <v>240</v>
-      </c>
-      <c r="AL27" t="s" s="2">
-        <v>241</v>
       </c>
       <c r="AM27" t="s" s="2">
         <v>74</v>
@@ -4471,7 +4467,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" t="s" s="2">
@@ -4479,31 +4475,31 @@
       </c>
       <c r="D28" s="2"/>
       <c r="E28" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="F28" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="G28" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="F28" t="s" s="2">
+      <c r="H28" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="I28" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="G28" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="H28" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="I28" t="s" s="2">
-        <v>84</v>
-      </c>
       <c r="J28" t="s" s="2">
+        <v>242</v>
+      </c>
+      <c r="K28" t="s" s="2">
         <v>243</v>
       </c>
-      <c r="K28" t="s" s="2">
+      <c r="L28" t="s" s="2">
         <v>244</v>
       </c>
-      <c r="L28" t="s" s="2">
+      <c r="M28" t="s" s="2">
         <v>245</v>
-      </c>
-      <c r="M28" t="s" s="2">
-        <v>246</v>
       </c>
       <c r="N28" s="2"/>
       <c r="O28" t="s" s="2">
@@ -4529,58 +4525,58 @@
         <v>74</v>
       </c>
       <c r="W28" t="s" s="2">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="X28" s="2"/>
       <c r="Y28" t="s" s="2">
+        <v>246</v>
+      </c>
+      <c r="Z28" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AA28" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AB28" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AC28" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AD28" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AE28" t="s" s="2">
+        <v>241</v>
+      </c>
+      <c r="AF28" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AG28" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AH28" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AI28" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="AJ28" t="s" s="2">
         <v>247</v>
       </c>
-      <c r="Z28" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AA28" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AB28" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AC28" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AD28" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AE28" t="s" s="2">
-        <v>242</v>
-      </c>
-      <c r="AF28" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AG28" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH28" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AI28" t="s" s="2">
-        <v>95</v>
-      </c>
-      <c r="AJ28" t="s" s="2">
+      <c r="AK28" t="s" s="2">
         <v>248</v>
       </c>
-      <c r="AK28" t="s" s="2">
+      <c r="AL28" t="s" s="2">
         <v>249</v>
       </c>
-      <c r="AL28" t="s" s="2">
+      <c r="AM28" t="s" s="2">
         <v>250</v>
-      </c>
-      <c r="AM28" t="s" s="2">
-        <v>251</v>
       </c>
     </row>
     <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B29" s="2"/>
       <c r="C29" t="s" s="2">
@@ -4591,7 +4587,7 @@
         <v>75</v>
       </c>
       <c r="F29" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G29" t="s" s="2">
         <v>74</v>
@@ -4603,13 +4599,13 @@
         <v>74</v>
       </c>
       <c r="J29" t="s" s="2">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="K29" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="L29" t="s" s="2">
         <v>97</v>
-      </c>
-      <c r="L29" t="s" s="2">
-        <v>98</v>
       </c>
       <c r="M29" s="2"/>
       <c r="N29" s="2"/>
@@ -4660,25 +4656,25 @@
         <v>74</v>
       </c>
       <c r="AE29" t="s" s="2">
+        <v>98</v>
+      </c>
+      <c r="AF29" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AG29" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AH29" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AI29" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AJ29" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AK29" t="s" s="2">
         <v>99</v>
-      </c>
-      <c r="AF29" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AG29" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH29" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AI29" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AJ29" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AK29" t="s" s="2">
-        <v>100</v>
       </c>
       <c r="AL29" t="s" s="2">
         <v>74</v>
@@ -4689,11 +4685,11 @@
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B30" s="2"/>
       <c r="C30" t="s" s="2">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D30" s="2"/>
       <c r="E30" t="s" s="2">
@@ -4712,16 +4708,16 @@
         <v>74</v>
       </c>
       <c r="J30" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="K30" t="s" s="2">
         <v>103</v>
       </c>
-      <c r="K30" t="s" s="2">
+      <c r="L30" t="s" s="2">
         <v>104</v>
       </c>
-      <c r="L30" t="s" s="2">
+      <c r="M30" t="s" s="2">
         <v>105</v>
-      </c>
-      <c r="M30" t="s" s="2">
-        <v>106</v>
       </c>
       <c r="N30" s="2"/>
       <c r="O30" t="s" s="2">
@@ -4759,19 +4755,19 @@
         <v>74</v>
       </c>
       <c r="AA30" t="s" s="2">
+        <v>106</v>
+      </c>
+      <c r="AB30" t="s" s="2">
         <v>107</v>
       </c>
-      <c r="AB30" t="s" s="2">
+      <c r="AC30" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AD30" t="s" s="2">
         <v>108</v>
       </c>
-      <c r="AC30" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AD30" t="s" s="2">
+      <c r="AE30" t="s" s="2">
         <v>109</v>
-      </c>
-      <c r="AE30" t="s" s="2">
-        <v>110</v>
       </c>
       <c r="AF30" t="s" s="2">
         <v>75</v>
@@ -4783,13 +4779,13 @@
         <v>74</v>
       </c>
       <c r="AI30" t="s" s="2">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AJ30" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AK30" t="s" s="2">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="AL30" t="s" s="2">
         <v>74</v>
@@ -4800,7 +4796,7 @@
     </row>
     <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B31" s="2"/>
       <c r="C31" t="s" s="2">
@@ -4820,22 +4816,22 @@
         <v>74</v>
       </c>
       <c r="I31" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J31" t="s" s="2">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="K31" t="s" s="2">
+        <v>254</v>
+      </c>
+      <c r="L31" t="s" s="2">
         <v>255</v>
       </c>
-      <c r="L31" t="s" s="2">
+      <c r="M31" t="s" s="2">
         <v>256</v>
       </c>
-      <c r="M31" t="s" s="2">
+      <c r="N31" t="s" s="2">
         <v>257</v>
-      </c>
-      <c r="N31" t="s" s="2">
-        <v>258</v>
       </c>
       <c r="O31" t="s" s="2">
         <v>74</v>
@@ -4860,29 +4856,29 @@
         <v>74</v>
       </c>
       <c r="W31" t="s" s="2">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="X31" s="2"/>
       <c r="Y31" t="s" s="2">
+        <v>258</v>
+      </c>
+      <c r="Z31" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AA31" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AB31" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AC31" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AD31" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AE31" t="s" s="2">
         <v>259</v>
-      </c>
-      <c r="Z31" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AA31" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AB31" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AC31" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AD31" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AE31" t="s" s="2">
-        <v>260</v>
       </c>
       <c r="AF31" t="s" s="2">
         <v>75</v>
@@ -4894,24 +4890,24 @@
         <v>74</v>
       </c>
       <c r="AI31" t="s" s="2">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="AJ31" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AK31" t="s" s="2">
+        <v>260</v>
+      </c>
+      <c r="AL31" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AM31" t="s" s="2">
         <v>261</v>
-      </c>
-      <c r="AL31" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AM31" t="s" s="2">
-        <v>262</v>
       </c>
     </row>
     <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B32" s="2"/>
       <c r="C32" t="s" s="2">
@@ -4922,31 +4918,31 @@
         <v>75</v>
       </c>
       <c r="F32" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="G32" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="H32" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="I32" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="G32" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="H32" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="I32" t="s" s="2">
-        <v>84</v>
-      </c>
       <c r="J32" t="s" s="2">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="K32" t="s" s="2">
+        <v>263</v>
+      </c>
+      <c r="L32" t="s" s="2">
         <v>264</v>
       </c>
-      <c r="L32" t="s" s="2">
+      <c r="M32" t="s" s="2">
         <v>265</v>
       </c>
-      <c r="M32" t="s" s="2">
+      <c r="N32" t="s" s="2">
         <v>266</v>
-      </c>
-      <c r="N32" t="s" s="2">
-        <v>267</v>
       </c>
       <c r="O32" t="s" s="2">
         <v>74</v>
@@ -4995,36 +4991,36 @@
         <v>74</v>
       </c>
       <c r="AE32" t="s" s="2">
+        <v>267</v>
+      </c>
+      <c r="AF32" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AG32" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AH32" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AI32" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="AJ32" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AK32" t="s" s="2">
         <v>268</v>
       </c>
-      <c r="AF32" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AG32" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH32" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AI32" t="s" s="2">
-        <v>95</v>
-      </c>
-      <c r="AJ32" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AK32" t="s" s="2">
+      <c r="AL32" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AM32" t="s" s="2">
         <v>269</v>
-      </c>
-      <c r="AL32" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AM32" t="s" s="2">
-        <v>270</v>
       </c>
     </row>
     <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B33" s="2"/>
       <c r="C33" t="s" s="2">
@@ -5035,28 +5031,28 @@
         <v>75</v>
       </c>
       <c r="F33" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="G33" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="H33" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="G33" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="H33" t="s" s="2">
-        <v>84</v>
-      </c>
       <c r="I33" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J33" t="s" s="2">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K33" t="s" s="2">
+        <v>271</v>
+      </c>
+      <c r="L33" t="s" s="2">
         <v>272</v>
       </c>
-      <c r="L33" t="s" s="2">
+      <c r="M33" t="s" s="2">
         <v>273</v>
-      </c>
-      <c r="M33" t="s" s="2">
-        <v>274</v>
       </c>
       <c r="N33" s="2"/>
       <c r="O33" t="s" s="2">
@@ -5082,49 +5078,49 @@
         <v>74</v>
       </c>
       <c r="W33" t="s" s="2">
+        <v>274</v>
+      </c>
+      <c r="X33" t="s" s="2">
         <v>275</v>
       </c>
-      <c r="X33" t="s" s="2">
+      <c r="Y33" t="s" s="2">
         <v>276</v>
       </c>
-      <c r="Y33" t="s" s="2">
+      <c r="Z33" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AA33" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AB33" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AC33" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AD33" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AE33" t="s" s="2">
+        <v>270</v>
+      </c>
+      <c r="AF33" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AG33" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AH33" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AI33" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="AJ33" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AK33" t="s" s="2">
         <v>277</v>
-      </c>
-      <c r="Z33" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AA33" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AB33" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AC33" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AD33" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AE33" t="s" s="2">
-        <v>271</v>
-      </c>
-      <c r="AF33" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AG33" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH33" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AI33" t="s" s="2">
-        <v>95</v>
-      </c>
-      <c r="AJ33" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AK33" t="s" s="2">
-        <v>278</v>
       </c>
       <c r="AL33" t="s" s="2">
         <v>74</v>
@@ -5135,7 +5131,7 @@
     </row>
     <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B34" s="2"/>
       <c r="C34" t="s" s="2">
@@ -5146,25 +5142,25 @@
         <v>75</v>
       </c>
       <c r="F34" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="G34" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="H34" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="I34" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="G34" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="H34" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="I34" t="s" s="2">
-        <v>84</v>
-      </c>
       <c r="J34" t="s" s="2">
+        <v>279</v>
+      </c>
+      <c r="K34" t="s" s="2">
         <v>280</v>
       </c>
-      <c r="K34" t="s" s="2">
+      <c r="L34" t="s" s="2">
         <v>281</v>
-      </c>
-      <c r="L34" t="s" s="2">
-        <v>282</v>
       </c>
       <c r="M34" s="2"/>
       <c r="N34" s="2"/>
@@ -5215,36 +5211,36 @@
         <v>74</v>
       </c>
       <c r="AE34" t="s" s="2">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="AF34" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AG34" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AH34" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AI34" t="s" s="2">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="AJ34" t="s" s="2">
+        <v>282</v>
+      </c>
+      <c r="AK34" t="s" s="2">
         <v>283</v>
       </c>
-      <c r="AK34" t="s" s="2">
+      <c r="AL34" t="s" s="2">
         <v>284</v>
       </c>
-      <c r="AL34" t="s" s="2">
+      <c r="AM34" t="s" s="2">
         <v>285</v>
-      </c>
-      <c r="AM34" t="s" s="2">
-        <v>286</v>
       </c>
     </row>
     <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B35" s="2"/>
       <c r="C35" t="s" s="2">
@@ -5255,7 +5251,7 @@
         <v>75</v>
       </c>
       <c r="F35" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G35" t="s" s="2">
         <v>74</v>
@@ -5267,16 +5263,16 @@
         <v>74</v>
       </c>
       <c r="J35" t="s" s="2">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="K35" t="s" s="2">
+        <v>287</v>
+      </c>
+      <c r="L35" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="L35" t="s" s="2">
+      <c r="M35" t="s" s="2">
         <v>289</v>
-      </c>
-      <c r="M35" t="s" s="2">
-        <v>290</v>
       </c>
       <c r="N35" s="2"/>
       <c r="O35" t="s" s="2">
@@ -5302,60 +5298,60 @@
         <v>74</v>
       </c>
       <c r="W35" t="s" s="2">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="X35" t="s" s="2">
+        <v>290</v>
+      </c>
+      <c r="Y35" t="s" s="2">
         <v>291</v>
       </c>
-      <c r="Y35" t="s" s="2">
+      <c r="Z35" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AA35" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AB35" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AC35" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AD35" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AE35" t="s" s="2">
+        <v>286</v>
+      </c>
+      <c r="AF35" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AG35" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AH35" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AI35" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="AJ35" t="s" s="2">
         <v>292</v>
       </c>
-      <c r="Z35" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AA35" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AB35" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AC35" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AD35" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AE35" t="s" s="2">
-        <v>287</v>
-      </c>
-      <c r="AF35" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AG35" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH35" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AI35" t="s" s="2">
-        <v>95</v>
-      </c>
-      <c r="AJ35" t="s" s="2">
+      <c r="AK35" t="s" s="2">
         <v>293</v>
       </c>
-      <c r="AK35" t="s" s="2">
+      <c r="AL35" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AM35" t="s" s="2">
         <v>294</v>
-      </c>
-      <c r="AL35" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AM35" t="s" s="2">
-        <v>295</v>
       </c>
     </row>
     <row r="36" hidden="true">
       <c r="A36" t="s" s="2">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B36" s="2"/>
       <c r="C36" t="s" s="2">
@@ -5366,25 +5362,25 @@
         <v>75</v>
       </c>
       <c r="F36" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="G36" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="H36" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="I36" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="G36" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="H36" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="I36" t="s" s="2">
-        <v>84</v>
-      </c>
       <c r="J36" t="s" s="2">
+        <v>296</v>
+      </c>
+      <c r="K36" t="s" s="2">
         <v>297</v>
       </c>
-      <c r="K36" t="s" s="2">
+      <c r="L36" t="s" s="2">
         <v>298</v>
-      </c>
-      <c r="L36" t="s" s="2">
-        <v>299</v>
       </c>
       <c r="M36" s="2"/>
       <c r="N36" s="2"/>
@@ -5435,25 +5431,25 @@
         <v>74</v>
       </c>
       <c r="AE36" t="s" s="2">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="AF36" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AG36" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AH36" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AI36" t="s" s="2">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="AJ36" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AK36" t="s" s="2">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="AL36" t="s" s="2">
         <v>74</v>
@@ -5464,7 +5460,7 @@
     </row>
     <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B37" s="2"/>
       <c r="C37" t="s" s="2">
@@ -5487,16 +5483,16 @@
         <v>74</v>
       </c>
       <c r="J37" t="s" s="2">
+        <v>301</v>
+      </c>
+      <c r="K37" t="s" s="2">
         <v>302</v>
       </c>
-      <c r="K37" t="s" s="2">
+      <c r="L37" t="s" s="2">
         <v>303</v>
       </c>
-      <c r="L37" t="s" s="2">
+      <c r="M37" t="s" s="2">
         <v>304</v>
-      </c>
-      <c r="M37" t="s" s="2">
-        <v>305</v>
       </c>
       <c r="N37" s="2"/>
       <c r="O37" t="s" s="2">
@@ -5546,7 +5542,7 @@
         <v>74</v>
       </c>
       <c r="AE37" t="s" s="2">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="AF37" t="s" s="2">
         <v>75</v>
@@ -5558,13 +5554,13 @@
         <v>74</v>
       </c>
       <c r="AI37" t="s" s="2">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="AJ37" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AK37" t="s" s="2">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="AL37" t="s" s="2">
         <v>74</v>
@@ -5575,7 +5571,7 @@
     </row>
     <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B38" s="2"/>
       <c r="C38" t="s" s="2">
@@ -5586,7 +5582,7 @@
         <v>75</v>
       </c>
       <c r="F38" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G38" t="s" s="2">
         <v>74</v>
@@ -5598,13 +5594,13 @@
         <v>74</v>
       </c>
       <c r="J38" t="s" s="2">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="K38" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="L38" t="s" s="2">
         <v>97</v>
-      </c>
-      <c r="L38" t="s" s="2">
-        <v>98</v>
       </c>
       <c r="M38" s="2"/>
       <c r="N38" s="2"/>
@@ -5655,25 +5651,25 @@
         <v>74</v>
       </c>
       <c r="AE38" t="s" s="2">
+        <v>98</v>
+      </c>
+      <c r="AF38" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AG38" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AH38" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AI38" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AJ38" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AK38" t="s" s="2">
         <v>99</v>
-      </c>
-      <c r="AF38" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AG38" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH38" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AI38" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AJ38" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AK38" t="s" s="2">
-        <v>100</v>
       </c>
       <c r="AL38" t="s" s="2">
         <v>74</v>
@@ -5684,11 +5680,11 @@
     </row>
     <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B39" s="2"/>
       <c r="C39" t="s" s="2">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D39" s="2"/>
       <c r="E39" t="s" s="2">
@@ -5707,16 +5703,16 @@
         <v>74</v>
       </c>
       <c r="J39" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="K39" t="s" s="2">
         <v>103</v>
       </c>
-      <c r="K39" t="s" s="2">
+      <c r="L39" t="s" s="2">
         <v>104</v>
       </c>
-      <c r="L39" t="s" s="2">
+      <c r="M39" t="s" s="2">
         <v>105</v>
-      </c>
-      <c r="M39" t="s" s="2">
-        <v>106</v>
       </c>
       <c r="N39" s="2"/>
       <c r="O39" t="s" s="2">
@@ -5766,7 +5762,7 @@
         <v>74</v>
       </c>
       <c r="AE39" t="s" s="2">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="AF39" t="s" s="2">
         <v>75</v>
@@ -5778,13 +5774,13 @@
         <v>74</v>
       </c>
       <c r="AI39" t="s" s="2">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AJ39" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AK39" t="s" s="2">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="AL39" t="s" s="2">
         <v>74</v>
@@ -5795,11 +5791,11 @@
     </row>
     <row r="40" hidden="true">
       <c r="A40" t="s" s="2">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B40" s="2"/>
       <c r="C40" t="s" s="2">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="D40" s="2"/>
       <c r="E40" t="s" s="2">
@@ -5812,25 +5808,25 @@
         <v>74</v>
       </c>
       <c r="H40" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I40" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J40" t="s" s="2">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="K40" t="s" s="2">
+        <v>310</v>
+      </c>
+      <c r="L40" t="s" s="2">
         <v>311</v>
       </c>
-      <c r="L40" t="s" s="2">
-        <v>312</v>
-      </c>
       <c r="M40" t="s" s="2">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="N40" t="s" s="2">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="O40" t="s" s="2">
         <v>74</v>
@@ -5879,7 +5875,7 @@
         <v>74</v>
       </c>
       <c r="AE40" t="s" s="2">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="AF40" t="s" s="2">
         <v>75</v>
@@ -5891,13 +5887,13 @@
         <v>74</v>
       </c>
       <c r="AI40" t="s" s="2">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AJ40" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AK40" t="s" s="2">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="AL40" t="s" s="2">
         <v>74</v>
@@ -5908,7 +5904,7 @@
     </row>
     <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B41" s="2"/>
       <c r="C41" t="s" s="2">
@@ -5916,10 +5912,10 @@
       </c>
       <c r="D41" s="2"/>
       <c r="E41" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F41" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G41" t="s" s="2">
         <v>74</v>
@@ -5931,17 +5927,17 @@
         <v>74</v>
       </c>
       <c r="J41" t="s" s="2">
+        <v>314</v>
+      </c>
+      <c r="K41" t="s" s="2">
         <v>315</v>
       </c>
-      <c r="K41" t="s" s="2">
+      <c r="L41" t="s" s="2">
         <v>316</v>
-      </c>
-      <c r="L41" t="s" s="2">
-        <v>317</v>
       </c>
       <c r="M41" s="2"/>
       <c r="N41" t="s" s="2">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="O41" t="s" s="2">
         <v>74</v>
@@ -5990,36 +5986,36 @@
         <v>74</v>
       </c>
       <c r="AE41" t="s" s="2">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AG41" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AH41" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AI41" t="s" s="2">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="AJ41" t="s" s="2">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="AK41" t="s" s="2">
+        <v>318</v>
+      </c>
+      <c r="AL41" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AM41" t="s" s="2">
         <v>319</v>
-      </c>
-      <c r="AL41" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AM41" t="s" s="2">
-        <v>320</v>
       </c>
     </row>
     <row r="42" hidden="true">
       <c r="A42" t="s" s="2">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B42" s="2"/>
       <c r="C42" t="s" s="2">
@@ -6030,7 +6026,7 @@
         <v>75</v>
       </c>
       <c r="F42" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G42" t="s" s="2">
         <v>74</v>
@@ -6042,17 +6038,17 @@
         <v>74</v>
       </c>
       <c r="J42" t="s" s="2">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K42" t="s" s="2">
+        <v>321</v>
+      </c>
+      <c r="L42" t="s" s="2">
         <v>322</v>
-      </c>
-      <c r="L42" t="s" s="2">
-        <v>323</v>
       </c>
       <c r="M42" s="2"/>
       <c r="N42" t="s" s="2">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="O42" t="s" s="2">
         <v>74</v>
@@ -6101,25 +6097,25 @@
         <v>74</v>
       </c>
       <c r="AE42" t="s" s="2">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="AF42" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AG42" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AH42" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AI42" t="s" s="2">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="AJ42" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AK42" t="s" s="2">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="AL42" t="s" s="2">
         <v>74</v>
@@ -6130,7 +6126,7 @@
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B43" s="2"/>
       <c r="C43" t="s" s="2">
@@ -6141,7 +6137,7 @@
         <v>75</v>
       </c>
       <c r="F43" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G43" t="s" s="2">
         <v>74</v>
@@ -6153,13 +6149,13 @@
         <v>74</v>
       </c>
       <c r="J43" t="s" s="2">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K43" t="s" s="2">
+        <v>326</v>
+      </c>
+      <c r="L43" t="s" s="2">
         <v>327</v>
-      </c>
-      <c r="L43" t="s" s="2">
-        <v>328</v>
       </c>
       <c r="M43" s="2"/>
       <c r="N43" s="2"/>
@@ -6210,36 +6206,36 @@
         <v>74</v>
       </c>
       <c r="AE43" t="s" s="2">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="AF43" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AG43" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AH43" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AI43" t="s" s="2">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="AJ43" t="s" s="2">
+        <v>328</v>
+      </c>
+      <c r="AK43" t="s" s="2">
+        <v>299</v>
+      </c>
+      <c r="AL43" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AM43" t="s" s="2">
         <v>329</v>
-      </c>
-      <c r="AK43" t="s" s="2">
-        <v>300</v>
-      </c>
-      <c r="AL43" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AM43" t="s" s="2">
-        <v>330</v>
       </c>
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B44" s="2"/>
       <c r="C44" t="s" s="2">
@@ -6250,7 +6246,7 @@
         <v>75</v>
       </c>
       <c r="F44" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G44" t="s" s="2">
         <v>74</v>
@@ -6262,13 +6258,13 @@
         <v>74</v>
       </c>
       <c r="J44" t="s" s="2">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="K44" t="s" s="2">
+        <v>331</v>
+      </c>
+      <c r="L44" t="s" s="2">
         <v>332</v>
-      </c>
-      <c r="L44" t="s" s="2">
-        <v>333</v>
       </c>
       <c r="M44" s="2"/>
       <c r="N44" s="2"/>
@@ -6319,25 +6315,25 @@
         <v>74</v>
       </c>
       <c r="AE44" t="s" s="2">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="AF44" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AG44" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AH44" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AI44" t="s" s="2">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="AJ44" t="s" s="2">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="AK44" t="s" s="2">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="AL44" t="s" s="2">
         <v>74</v>
@@ -6348,7 +6344,7 @@
     </row>
     <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B45" s="2"/>
       <c r="C45" t="s" s="2">
@@ -6359,7 +6355,7 @@
         <v>75</v>
       </c>
       <c r="F45" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G45" t="s" s="2">
         <v>74</v>
@@ -6371,13 +6367,13 @@
         <v>74</v>
       </c>
       <c r="J45" t="s" s="2">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="K45" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="L45" t="s" s="2">
         <v>97</v>
-      </c>
-      <c r="L45" t="s" s="2">
-        <v>98</v>
       </c>
       <c r="M45" s="2"/>
       <c r="N45" s="2"/>
@@ -6428,25 +6424,25 @@
         <v>74</v>
       </c>
       <c r="AE45" t="s" s="2">
+        <v>98</v>
+      </c>
+      <c r="AF45" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AG45" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AH45" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AI45" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AJ45" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AK45" t="s" s="2">
         <v>99</v>
-      </c>
-      <c r="AF45" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AG45" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH45" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AI45" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AJ45" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AK45" t="s" s="2">
-        <v>100</v>
       </c>
       <c r="AL45" t="s" s="2">
         <v>74</v>
@@ -6457,11 +6453,11 @@
     </row>
     <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B46" s="2"/>
       <c r="C46" t="s" s="2">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D46" s="2"/>
       <c r="E46" t="s" s="2">
@@ -6480,16 +6476,16 @@
         <v>74</v>
       </c>
       <c r="J46" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="K46" t="s" s="2">
         <v>103</v>
       </c>
-      <c r="K46" t="s" s="2">
+      <c r="L46" t="s" s="2">
         <v>104</v>
       </c>
-      <c r="L46" t="s" s="2">
+      <c r="M46" t="s" s="2">
         <v>105</v>
-      </c>
-      <c r="M46" t="s" s="2">
-        <v>106</v>
       </c>
       <c r="N46" s="2"/>
       <c r="O46" t="s" s="2">
@@ -6539,7 +6535,7 @@
         <v>74</v>
       </c>
       <c r="AE46" t="s" s="2">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="AF46" t="s" s="2">
         <v>75</v>
@@ -6551,13 +6547,13 @@
         <v>74</v>
       </c>
       <c r="AI46" t="s" s="2">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AJ46" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AK46" t="s" s="2">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="AL46" t="s" s="2">
         <v>74</v>
@@ -6568,11 +6564,11 @@
     </row>
     <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B47" s="2"/>
       <c r="C47" t="s" s="2">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="D47" s="2"/>
       <c r="E47" t="s" s="2">
@@ -6585,25 +6581,25 @@
         <v>74</v>
       </c>
       <c r="H47" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I47" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J47" t="s" s="2">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="K47" t="s" s="2">
+        <v>310</v>
+      </c>
+      <c r="L47" t="s" s="2">
         <v>311</v>
       </c>
-      <c r="L47" t="s" s="2">
-        <v>312</v>
-      </c>
       <c r="M47" t="s" s="2">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="N47" t="s" s="2">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="O47" t="s" s="2">
         <v>74</v>
@@ -6652,7 +6648,7 @@
         <v>74</v>
       </c>
       <c r="AE47" t="s" s="2">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="AF47" t="s" s="2">
         <v>75</v>
@@ -6664,13 +6660,13 @@
         <v>74</v>
       </c>
       <c r="AI47" t="s" s="2">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AJ47" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AK47" t="s" s="2">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="AL47" t="s" s="2">
         <v>74</v>
@@ -6681,7 +6677,7 @@
     </row>
     <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B48" s="2"/>
       <c r="C48" t="s" s="2">
@@ -6692,7 +6688,7 @@
         <v>75</v>
       </c>
       <c r="F48" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G48" t="s" s="2">
         <v>74</v>
@@ -6704,13 +6700,13 @@
         <v>74</v>
       </c>
       <c r="J48" t="s" s="2">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="K48" t="s" s="2">
+        <v>338</v>
+      </c>
+      <c r="L48" t="s" s="2">
         <v>339</v>
-      </c>
-      <c r="L48" t="s" s="2">
-        <v>340</v>
       </c>
       <c r="M48" s="2"/>
       <c r="N48" s="2"/>
@@ -6761,36 +6757,36 @@
         <v>74</v>
       </c>
       <c r="AE48" t="s" s="2">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="AF48" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AG48" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AH48" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AI48" t="s" s="2">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="AJ48" t="s" s="2">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="AK48" t="s" s="2">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="AL48" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AM48" t="s" s="2">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="49" hidden="true">
       <c r="A49" t="s" s="2">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B49" s="2"/>
       <c r="C49" t="s" s="2">
@@ -6801,7 +6797,7 @@
         <v>75</v>
       </c>
       <c r="F49" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G49" t="s" s="2">
         <v>74</v>
@@ -6813,13 +6809,13 @@
         <v>74</v>
       </c>
       <c r="J49" t="s" s="2">
+        <v>342</v>
+      </c>
+      <c r="K49" t="s" s="2">
         <v>343</v>
       </c>
-      <c r="K49" t="s" s="2">
+      <c r="L49" t="s" s="2">
         <v>344</v>
-      </c>
-      <c r="L49" t="s" s="2">
-        <v>345</v>
       </c>
       <c r="M49" s="2"/>
       <c r="N49" s="2"/>
@@ -6870,31 +6866,31 @@
         <v>74</v>
       </c>
       <c r="AE49" t="s" s="2">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AF49" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AG49" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AH49" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AI49" t="s" s="2">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="AJ49" t="s" s="2">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="AK49" t="s" s="2">
+        <v>345</v>
+      </c>
+      <c r="AL49" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AM49" t="s" s="2">
         <v>346</v>
-      </c>
-      <c r="AL49" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AM49" t="s" s="2">
-        <v>347</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added cytogenetics profile and example
</commit_message>
<xml_diff>
--- a/docs/StructureDefinition-cibmtr-additional-peri-transplant-medication.xlsx
+++ b/docs/StructureDefinition-cibmtr-additional-peri-transplant-medication.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2022-11-09T14:05:34-06:00</t>
+    <t>2022-11-10T14:39:35-06:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -500,7 +500,7 @@
     <t>Need to be unambiguous about the source of the definition of the symbol.</t>
   </si>
   <si>
-    <t>http://terminology.nmdp.org/codesystem/transplant-center</t>
+    <t>http://terminology.cibmtr.org/codesystem/transplant-center</t>
   </si>
   <si>
     <t>Coding.system</t>

</xml_diff>

<commit_message>
updated footer background color
</commit_message>
<xml_diff>
--- a/docs/StructureDefinition-cibmtr-additional-peri-transplant-medication.xlsx
+++ b/docs/StructureDefinition-cibmtr-additional-peri-transplant-medication.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-05-04T09:48:28-05:00</t>
+    <t>2023-05-04T21:27:58-05:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1454,17 +1454,17 @@
   <dimension ref="A1:AN49"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="52.19921875" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="37.84765625" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="16.578125" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="4" max="4" width="38.81640625" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="5" max="5" width="5.8984375" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="4.69921875" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="5.07421875" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" width="14.625" customWidth="true" bestFit="true"/>
-    <col min="9" max="9" width="11.98828125" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="51.0703125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="37.21875" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="16.44140625" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="4" max="4" width="38.4609375" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="5" max="5" width="6.1484375" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="4.58203125" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="4.94140625" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="14.7109375" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="12.1875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="31.81640625" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="30.390625" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -1473,25 +1473,25 @@
     <col min="17" max="17" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="18" max="18" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="19" max="19" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="20" max="20" width="8.84375" customWidth="true" bestFit="true"/>
-    <col min="21" max="21" width="15.7109375" customWidth="true" bestFit="true"/>
-    <col min="22" max="22" width="16.0859375" customWidth="true" bestFit="true"/>
-    <col min="23" max="23" width="17.078125" customWidth="true" bestFit="true"/>
-    <col min="24" max="24" width="16.30859375" customWidth="true" bestFit="true"/>
-    <col min="25" max="25" width="95.77734375" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="75.94140625" customWidth="true" bestFit="true"/>
-    <col min="27" max="27" width="5.69140625" customWidth="true" bestFit="true"/>
-    <col min="28" max="28" width="19.73046875" customWidth="true" bestFit="true"/>
-    <col min="29" max="29" width="40.0390625" customWidth="true" bestFit="true"/>
-    <col min="30" max="30" width="14.984375" customWidth="true" bestFit="true"/>
-    <col min="31" max="31" width="12.30078125" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="32" max="32" width="34.0703125" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="33" max="33" width="9.5" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="34" max="34" width="9.875" customWidth="true" bestFit="true"/>
+    <col min="20" max="20" width="9.04296875" customWidth="true" bestFit="true"/>
+    <col min="21" max="21" width="15.77734375" customWidth="true" bestFit="true"/>
+    <col min="22" max="22" width="16.13671875" customWidth="true" bestFit="true"/>
+    <col min="23" max="23" width="17.40234375" customWidth="true" bestFit="true"/>
+    <col min="24" max="24" width="16.9609375" customWidth="true" bestFit="true"/>
+    <col min="25" max="25" width="95.2265625" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="77.71875" customWidth="true" bestFit="true"/>
+    <col min="27" max="27" width="5.8828125" customWidth="true" bestFit="true"/>
+    <col min="28" max="28" width="20.84375" customWidth="true" bestFit="true"/>
+    <col min="29" max="29" width="40.0859375" customWidth="true" bestFit="true"/>
+    <col min="30" max="30" width="15.703125" customWidth="true" bestFit="true"/>
+    <col min="31" max="31" width="13.125" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="32" max="32" width="33.4296875" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="33" max="33" width="9.53125" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="34" max="34" width="9.890625" customWidth="true" bestFit="true"/>
     <col min="35" max="35" width="100.703125" customWidth="true"/>
-    <col min="37" max="37" width="195.390625" customWidth="true" bestFit="true"/>
-    <col min="38" max="38" width="95.72265625" customWidth="true" bestFit="true"/>
-    <col min="39" max="39" width="32.84375" customWidth="true" bestFit="true"/>
+    <col min="37" max="37" width="194.96484375" customWidth="true" bestFit="true"/>
+    <col min="38" max="38" width="95.25" customWidth="true" bestFit="true"/>
+    <col min="39" max="39" width="33.05078125" customWidth="true" bestFit="true"/>
     <col min="40" max="40" width="255.0" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>

</xml_diff>